<commit_message>
agrega mapas y capas
</commit_message>
<xml_diff>
--- a/data/data/Capacidad de almacenamiento al 2019.xlsx
+++ b/data/data/Capacidad de almacenamiento al 2019.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\planInfra\data\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F66CF01E-B447-4587-B34B-771B98C27346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00E60EDA-3FE2-4D77-B7A3-7593F178550C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="1" xr2:uid="{00E60EDA-3FE2-4D77-B7A3-7593F178550C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -296,12 +296,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -655,482 +654,482 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" style="2"/>
+    <col min="4" max="4" width="11.5703125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="3">
         <v>73</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="3">
         <v>0</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="3">
         <v>340</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="3">
         <v>990</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>22</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="3">
         <v>10</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="3">
         <v>163</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="3">
         <v>5</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>168</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <v>116</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6" s="3">
         <v>36</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>152</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="3">
         <v>23</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="3">
         <v>0</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="3">
         <v>490</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="3">
         <v>256</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="3">
         <v>746</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="3">
         <v>434</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="3">
         <v>78</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="3">
         <v>9</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="3">
         <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="3">
         <v>923</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="3">
         <v>28</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="3">
         <v>951</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="3">
         <v>585</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="3" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="3">
         <v>139</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="3">
         <v>47</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="3">
         <v>186</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="3">
         <v>158</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C14" s="3">
         <v>30</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="3">
         <v>188</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C15" s="3">
         <v>494</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="3">
         <v>283</v>
       </c>
-      <c r="C16" s="4">
+      <c r="C16" s="3">
         <v>5</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="3">
         <v>288</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C17" s="3">
         <v>428</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="3" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="3">
         <v>247</v>
       </c>
-      <c r="C18" s="4">
+      <c r="C18" s="3">
         <v>143</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="3">
         <v>390</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="3">
         <v>296</v>
       </c>
-      <c r="C19" s="4">
+      <c r="C19" s="3">
         <v>201</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="3">
         <v>497</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B20" s="3">
         <v>163</v>
       </c>
-      <c r="C20" s="4">
+      <c r="C20" s="3">
         <v>8</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="3">
         <v>171</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="4">
+      <c r="B21" s="3">
         <v>28</v>
       </c>
-      <c r="C21" s="4">
+      <c r="C21" s="3">
         <v>35</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="3">
         <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B22" s="4">
+      <c r="B22" s="3">
         <v>667</v>
       </c>
-      <c r="C22" s="4">
+      <c r="C22" s="3">
         <v>48</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D22" s="3">
         <v>715</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="4">
+      <c r="B23" s="3">
         <v>265</v>
       </c>
-      <c r="C23" s="4">
+      <c r="C23" s="3">
         <v>35</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="3">
         <v>301</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="4">
+      <c r="B24" s="3">
         <v>0</v>
       </c>
-      <c r="C24" s="4">
+      <c r="C24" s="3">
         <v>0</v>
       </c>
-      <c r="D24" s="4">
+      <c r="D24" s="3">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B25" s="4">
+      <c r="B25" s="3">
         <v>71</v>
       </c>
-      <c r="C25" s="4">
+      <c r="C25" s="3">
         <v>7</v>
       </c>
-      <c r="D25" s="4">
+      <c r="D25" s="3">
         <v>77</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C26" s="4">
+      <c r="C26" s="3">
         <v>629</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="3" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="3" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B28" s="4">
+      <c r="B28" s="3">
         <v>50</v>
       </c>
-      <c r="C28" s="4">
+      <c r="C28" s="3">
         <v>0</v>
       </c>
-      <c r="D28" s="4">
+      <c r="D28" s="3">
         <v>50</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C29" s="4">
+      <c r="C29" s="3">
         <v>297</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="3" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B30" s="4">
+      <c r="B30" s="3">
         <v>375</v>
       </c>
-      <c r="C30" s="4">
+      <c r="C30" s="3">
         <v>40</v>
       </c>
-      <c r="D30" s="4">
+      <c r="D30" s="3">
         <v>415</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B31" s="4">
+      <c r="B31" s="3">
         <v>661</v>
       </c>
-      <c r="C31" s="4">
+      <c r="C31" s="3">
         <v>10</v>
       </c>
-      <c r="D31" s="4">
+      <c r="D31" s="3">
         <v>670</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B32" s="4">
+      <c r="B32" s="3">
         <v>341</v>
       </c>
-      <c r="C32" s="4">
+      <c r="C32" s="3">
         <v>0</v>
       </c>
-      <c r="D32" s="4">
+      <c r="D32" s="3">
         <v>341</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
+      <c r="A33" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B33" s="4">
+      <c r="B33" s="3">
         <v>900</v>
       </c>
-      <c r="C33" s="4">
+      <c r="C33" s="3">
         <v>20</v>
       </c>
-      <c r="D33" s="4">
+      <c r="D33" s="3">
         <v>919</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="7" t="s">
+      <c r="A34" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="4" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>